<commit_message>
e-codices workflow überarbeitet und neu strukturiert.
</commit_message>
<xml_diff>
--- a/e-codices/e-codices.xlsx
+++ b/e-codices/e-codices.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HeimK\switchdrive\dlza\dlza\e-codices\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9F5C030-D620-496A-AD2F-72827409B58A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42598114-2BEC-4D84-9626-064B45263E8B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19180" windowHeight="7940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -397,64 +397,64 @@
     <t>Anfang des 13. Jahrhunderts</t>
   </si>
   <si>
-    <t>9914249443205505x</t>
-  </si>
-  <si>
-    <t>9914249441205505x</t>
-  </si>
-  <si>
-    <t>9914249440305505x</t>
-  </si>
-  <si>
-    <t>9914249439505505x</t>
-  </si>
-  <si>
-    <t>9914249439005505x</t>
-  </si>
-  <si>
-    <t>9914249437805505x</t>
-  </si>
-  <si>
-    <t>9914249437605505x</t>
-  </si>
-  <si>
-    <t>9914249437405505x</t>
-  </si>
-  <si>
-    <t>9914249436205505x</t>
-  </si>
-  <si>
-    <t>9914249426405505x</t>
-  </si>
-  <si>
-    <t>9914249425905505x</t>
-  </si>
-  <si>
-    <t>9914249424805505x</t>
-  </si>
-  <si>
-    <t>9914249424605505x</t>
-  </si>
-  <si>
-    <t>9914249423805505x</t>
-  </si>
-  <si>
-    <t>9914249329905505x</t>
-  </si>
-  <si>
-    <t>9914249303805505x</t>
-  </si>
-  <si>
-    <t>9914249300405505x</t>
-  </si>
-  <si>
-    <t>9914249327205505x</t>
-  </si>
-  <si>
-    <t>9914249325605505x</t>
-  </si>
-  <si>
-    <t>9914249327405505x</t>
+    <t>9914249443205505</t>
+  </si>
+  <si>
+    <t>9914249441205505</t>
+  </si>
+  <si>
+    <t>9914249440305505</t>
+  </si>
+  <si>
+    <t>9914249439505505</t>
+  </si>
+  <si>
+    <t>9914249439005505</t>
+  </si>
+  <si>
+    <t>9914249437805505</t>
+  </si>
+  <si>
+    <t>9914249437605505</t>
+  </si>
+  <si>
+    <t>9914249437405505</t>
+  </si>
+  <si>
+    <t>9914249436205505</t>
+  </si>
+  <si>
+    <t>9914249426405505</t>
+  </si>
+  <si>
+    <t>9914249425905505</t>
+  </si>
+  <si>
+    <t>9914249424805505</t>
+  </si>
+  <si>
+    <t>9914249424605505</t>
+  </si>
+  <si>
+    <t>9914249423805505</t>
+  </si>
+  <si>
+    <t>9914249329905505</t>
+  </si>
+  <si>
+    <t>9914249303805505</t>
+  </si>
+  <si>
+    <t>9914249300405505</t>
+  </si>
+  <si>
+    <t>9914249327205505</t>
+  </si>
+  <si>
+    <t>9914249325605505</t>
+  </si>
+  <si>
+    <t>9914249327405505</t>
   </si>
 </sst>
 </file>
@@ -944,7 +944,7 @@
       <c r="D2" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="4" t="s">
         <v>124</v>
       </c>
       <c r="F2" t="s">
@@ -968,7 +968,7 @@
       <c r="D3" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="4" t="s">
         <v>125</v>
       </c>
       <c r="F3" t="s">
@@ -991,7 +991,7 @@
       <c r="D4" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>126</v>
       </c>
       <c r="F4" t="s">
@@ -1014,7 +1014,7 @@
       <c r="D5" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="4" t="s">
         <v>127</v>
       </c>
       <c r="F5" t="s">
@@ -1037,7 +1037,7 @@
       <c r="D6" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="4" t="s">
         <v>128</v>
       </c>
       <c r="F6" t="s">
@@ -1060,7 +1060,7 @@
       <c r="D7" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="4" t="s">
         <v>129</v>
       </c>
       <c r="F7" t="s">
@@ -1083,7 +1083,7 @@
       <c r="D8" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="4" t="s">
         <v>130</v>
       </c>
       <c r="F8" t="s">
@@ -1106,7 +1106,7 @@
       <c r="D9" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="4" t="s">
         <v>131</v>
       </c>
       <c r="F9" t="s">
@@ -1129,7 +1129,7 @@
       <c r="D10" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="4" t="s">
         <v>132</v>
       </c>
       <c r="F10" s="3" t="s">
@@ -1153,7 +1153,7 @@
       <c r="D11" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="4" t="s">
         <v>133</v>
       </c>
       <c r="F11" t="s">
@@ -1176,7 +1176,7 @@
       <c r="D12" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="4" t="s">
         <v>134</v>
       </c>
       <c r="F12" t="s">
@@ -1199,7 +1199,7 @@
       <c r="D13" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="4" t="s">
         <v>135</v>
       </c>
       <c r="F13" t="s">
@@ -1222,7 +1222,7 @@
       <c r="D14" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="4" t="s">
         <v>136</v>
       </c>
       <c r="F14" t="s">
@@ -1245,7 +1245,7 @@
       <c r="D15" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="E15" s="4" t="s">
         <v>137</v>
       </c>
       <c r="F15" t="s">
@@ -1268,7 +1268,7 @@
       <c r="D16" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="E16" s="4" t="s">
         <v>138</v>
       </c>
       <c r="F16" t="s">
@@ -1291,7 +1291,7 @@
       <c r="D17" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="E17" s="4" t="s">
         <v>139</v>
       </c>
       <c r="F17" t="s">
@@ -1314,7 +1314,7 @@
       <c r="D18" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="E18" s="5" t="s">
+      <c r="E18" s="4" t="s">
         <v>140</v>
       </c>
       <c r="F18" t="s">
@@ -1338,7 +1338,7 @@
       <c r="D19" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E19" s="5" t="s">
+      <c r="E19" s="4" t="s">
         <v>141</v>
       </c>
       <c r="F19" t="s">
@@ -1361,7 +1361,7 @@
       <c r="D20" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="E20" s="4" t="s">
         <v>142</v>
       </c>
       <c r="F20" t="s">
@@ -1400,6 +1400,9 @@
   </sheetData>
   <autoFilter ref="A1:H21" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="E2:E21" numberStoredAsText="1"/>
+  </ignoredErrors>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>